<commit_message>
Added Ketty's notebook file
</commit_message>
<xml_diff>
--- a/Data/Data Dictionary.xlsx
+++ b/Data/Data Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rebeccaquaye/Complex Data Analytics/Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Documents\Daniels College of Business\Fall 2026\Complex Analytics\consumer-financial-complaints\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FDEB969-34F5-C64F-AC9D-C751C63ECB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{9DC70436-4C0B-9944-A2BF-6EF13F1A6E5E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9DC70436-4C0B-9944-A2BF-6EF13F1A6E5E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -621,7 +621,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE6511C-5D56-A842-B3A2-28B9E09060BB}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="36.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="36.33203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="29.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.5" customWidth="1"/>
@@ -629,7 +629,7 @@
     <col min="4" max="4" width="48.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="28" x14ac:dyDescent="0.65">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="4" t="s">
@@ -637,7 +637,7 @@
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" ht="21" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="20" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -651,7 +651,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -665,7 +665,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
@@ -679,7 +679,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="63" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
@@ -693,7 +693,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
@@ -707,7 +707,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
@@ -721,7 +721,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
         <v>21</v>
       </c>
@@ -735,7 +735,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
@@ -749,7 +749,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
         <v>29</v>
       </c>
@@ -763,7 +763,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>32</v>
       </c>
@@ -777,7 +777,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A12" s="5" t="s">
         <v>35</v>
       </c>
@@ -791,7 +791,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
         <v>37</v>
       </c>
@@ -805,7 +805,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -819,7 +819,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
         <v>42</v>
       </c>
@@ -833,7 +833,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
         <v>45</v>
       </c>
@@ -847,7 +847,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="63" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ht="61.5" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
         <v>48</v>
       </c>
@@ -861,7 +861,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="41" x14ac:dyDescent="0.45">
       <c r="A18" s="5" t="s">
         <v>52</v>
       </c>

</xml_diff>